<commit_message>
Analiz tablosuna para kazanma sonrası RPM sayfası
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC3abK5TfSXuseNg5SJgXH
</commit_message>
<xml_diff>
--- a/output/eli_holloway_analiz.xlsx
+++ b/output/eli_holloway_analiz.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="En İyi 20" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Haftalık İzlenme" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trafik &amp; Ülke" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RPM (24 Nis sonrası)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Videolar'!$A$1:$M$114</definedName>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="168" formatCode="DD.MM.YYYY"/>
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +54,9 @@
     <font>
       <color rgb="001F5FBF"/>
       <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -125,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -192,6 +196,7 @@
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1147,7 +1152,7 @@
     <row r="14">
       <c r="A14" s="51" t="inlineStr">
         <is>
-          <t>• RPM = 1.000 izlenme başına gelir. 200 izlenme altındaki videolar video sayfasında boş bırakıldı.</t>
+          <t>• RPM = 1.000 izlenme başına gelir. 24.04 öncesi yüklenen videoların RPM'i düşük görünür (para kazanma kapalıydı). Gerçek RPM için "RPM (24 Nis sonrası)" sayfasına bak.</t>
         </is>
       </c>
     </row>
@@ -8254,4 +8259,187 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Toplam izlenme</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>24 Nis sonrası izlenme</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Gelir $</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Gerçek RPM $</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="53" t="inlineStr">
+        <is>
+          <t>$3 Liquid Makes ANY Faded Car Look BRAND NEW. Detailers PRAYED You'd Never Find This</t>
+        </is>
+      </c>
+      <c r="B2" s="54" t="n">
+        <v>12392</v>
+      </c>
+      <c r="C2" s="54" t="n">
+        <v>1303</v>
+      </c>
+      <c r="D2" s="58" t="n">
+        <v>20.31</v>
+      </c>
+      <c r="E2" s="59" t="n">
+        <v>15.59</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="53" t="inlineStr">
+        <is>
+          <t>$2 Oil Makes ANY Engine Last FOREVER — Motor Industry PRAYED You'd Forget</t>
+        </is>
+      </c>
+      <c r="B3" s="54" t="n">
+        <v>20981</v>
+      </c>
+      <c r="C3" s="54" t="n">
+        <v>3142</v>
+      </c>
+      <c r="D3" s="58" t="n">
+        <v>35.84</v>
+      </c>
+      <c r="E3" s="59" t="n">
+        <v>11.41</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="53" t="inlineStr">
+        <is>
+          <t>$2 Oil Regrows ANY Hair In 30 Days — Pharma Industry BURIED This For 60 Years</t>
+        </is>
+      </c>
+      <c r="B4" s="54" t="n">
+        <v>56125</v>
+      </c>
+      <c r="C4" s="54" t="n">
+        <v>56125</v>
+      </c>
+      <c r="D4" s="58" t="n">
+        <v>419.75</v>
+      </c>
+      <c r="E4" s="59" t="n">
+        <v>7.48</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="53" t="inlineStr">
+        <is>
+          <t>This $2 Plant Repels EVERY Insect FOREVER — Chemical Industry Wants It Gone</t>
+        </is>
+      </c>
+      <c r="B5" s="54" t="n">
+        <v>46988</v>
+      </c>
+      <c r="C5" s="54" t="n">
+        <v>1223</v>
+      </c>
+      <c r="D5" s="58" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="E5" s="59" t="n">
+        <v>5.67</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="53" t="inlineStr">
+        <is>
+          <t>$2 Oil Makes ANY Leather Last 100 Years — Shoe Industry PRAYED You'd Forget</t>
+        </is>
+      </c>
+      <c r="B6" s="54" t="n">
+        <v>72171</v>
+      </c>
+      <c r="C6" s="54" t="n">
+        <v>10261</v>
+      </c>
+      <c r="D6" s="58" t="n">
+        <v>36.03</v>
+      </c>
+      <c r="E6" s="59" t="n">
+        <v>3.51</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="64" t="inlineStr">
+        <is>
+          <t>KANAL TOPLAMI</t>
+        </is>
+      </c>
+      <c r="B7" s="54" t="n">
+        <v>302969</v>
+      </c>
+      <c r="C7" s="54" t="n">
+        <v>105856</v>
+      </c>
+      <c r="D7" s="58" t="n">
+        <v>770.8200000000001</v>
+      </c>
+      <c r="E7" s="59" t="n">
+        <v>7.28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="51" t="inlineStr">
+        <is>
+          <t>Para kazanma 24.04.2026'da açıldı; toplam izlenmenin %65'i bundan önce geldi ve gelir üretmedi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="51" t="inlineStr">
+        <is>
+          <t>Gerçek RPM = gelir / para kazanma sonrası izlenme. Studio günlük kırılımı yalnızca bu 5 video için verdi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="51" t="inlineStr">
+        <is>
+          <t>Sonuç: araba/motor videoları en yüksek RPM ($11–16), sağlık $7.5, ev/temizlik $3.5–6.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>